<commit_message>
Fix duplicated California 2025 EV sales and refresh derived results
</commit_message>
<xml_diff>
--- a/Outputs/Recycling_Plot_Data/ACCII/01_Geofacet_StateMass_2050_data_ACCII.xlsx
+++ b/Outputs/Recycling_Plot_Data/ACCII/01_Geofacet_StateMass_2050_data_ACCII.xlsx
@@ -775,7 +775,7 @@
         <v>2050</v>
       </c>
       <c r="F15">
-        <v>0.3270303171332421</v>
+        <v>0.3267026060305782</v>
       </c>
     </row>
     <row r="16">
@@ -1111,7 +1111,7 @@
         <v>2050</v>
       </c>
       <c r="F27">
-        <v>0.1989434429227222</v>
+        <v>0.1987440853352683</v>
       </c>
     </row>
     <row r="28">
@@ -1139,7 +1139,7 @@
         <v>2050</v>
       </c>
       <c r="F28">
-        <v>0.4528003859610958</v>
+        <v>0.4523466429715445</v>
       </c>
     </row>
     <row r="29">
@@ -1419,7 +1419,7 @@
         <v>2050</v>
       </c>
       <c r="F38">
-        <v>1.827345491614864</v>
+        <v>1.813918989283646</v>
       </c>
     </row>
     <row r="39">
@@ -1447,7 +1447,7 @@
         <v>2050</v>
       </c>
       <c r="F39">
-        <v>1.122090972956097</v>
+        <v>1.120966546103993</v>
       </c>
     </row>
     <row r="40">
@@ -1475,7 +1475,7 @@
         <v>2050</v>
       </c>
       <c r="F40">
-        <v>0.03856747147089685</v>
+        <v>0.03852882371275174</v>
       </c>
     </row>
     <row r="41">
@@ -1503,7 +1503,7 @@
         <v>2050</v>
       </c>
       <c r="F41">
-        <v>1.090097985500247</v>
+        <v>1.079440083136078</v>
       </c>
     </row>
     <row r="42">
@@ -1643,7 +1643,7 @@
         <v>2050</v>
       </c>
       <c r="F46">
-        <v>0.005957899815277576</v>
+        <v>0.005951929512783481</v>
       </c>
     </row>
     <row r="47">
@@ -2315,7 +2315,7 @@
         <v>2050</v>
       </c>
       <c r="F70">
-        <v>0.01191579963055515</v>
+        <v>0.01190385902556696</v>
       </c>
     </row>
     <row r="71">
@@ -2455,7 +2455,7 @@
         <v>2050</v>
       </c>
       <c r="F75">
-        <v>1.253992796042612</v>
+        <v>1.252736192784766</v>
       </c>
     </row>
     <row r="76">
@@ -2483,7 +2483,7 @@
         <v>2050</v>
       </c>
       <c r="F76">
-        <v>1.088309699590704</v>
+        <v>1.087219124335116</v>
       </c>
     </row>
     <row r="77">
@@ -3127,7 +3127,7 @@
         <v>2050</v>
       </c>
       <c r="F99">
-        <v>0.09910009610098244</v>
+        <v>0.0990007897062358</v>
       </c>
     </row>
     <row r="100">
@@ -3155,7 +3155,7 @@
         <v>2050</v>
       </c>
       <c r="F100">
-        <v>0.7149479778333093</v>
+        <v>0.7142315415340178</v>
       </c>
     </row>
     <row r="101">
@@ -3295,7 +3295,7 @@
         <v>2050</v>
       </c>
       <c r="F105">
-        <v>0.3712289599942802</v>
+        <v>0.3708569582395593</v>
       </c>
     </row>
     <row r="106">
@@ -3323,7 +3323,7 @@
         <v>2050</v>
       </c>
       <c r="F106">
-        <v>0.8266387397037127</v>
+        <v>0.8258103801336653</v>
       </c>
     </row>
     <row r="107">
@@ -3491,7 +3491,7 @@
         <v>2050</v>
       </c>
       <c r="F112">
-        <v>0.2383159926111031</v>
+        <v>0.2380771805113393</v>
       </c>
     </row>
     <row r="113">
@@ -3631,7 +3631,7 @@
         <v>2050</v>
       </c>
       <c r="F117">
-        <v>0.5648705477755999</v>
+        <v>0.564304501325544</v>
       </c>
     </row>
     <row r="118">
@@ -3659,7 +3659,7 @@
         <v>2050</v>
       </c>
       <c r="F118">
-        <v>0.2065405269296227</v>
+        <v>0.2063335564431606</v>
       </c>
     </row>
     <row r="119">
@@ -3967,7 +3967,7 @@
         <v>2050</v>
       </c>
       <c r="F129">
-        <v>0.109039835739911</v>
+        <v>0.1089305689137712</v>
       </c>
     </row>
     <row r="130">
@@ -4331,7 +4331,7 @@
         <v>2050</v>
       </c>
       <c r="F142">
-        <v>0.001588773284074021</v>
+        <v>0.001587181203408928</v>
       </c>
     </row>
     <row r="143">
@@ -4639,7 +4639,7 @@
         <v>2050</v>
       </c>
       <c r="F153">
-        <v>2.013733772791184</v>
+        <v>2.011715846988653</v>
       </c>
     </row>
     <row r="154">
@@ -4667,7 +4667,7 @@
         <v>2050</v>
       </c>
       <c r="F154">
-        <v>1.283172742882382</v>
+        <v>1.281886898933221</v>
       </c>
     </row>
     <row r="155">
@@ -5003,7 +5003,7 @@
         <v>2050</v>
       </c>
       <c r="F166">
-        <v>0.001588773284074021</v>
+        <v>0.001587181203408928</v>
       </c>
     </row>
     <row r="167">
@@ -5171,7 +5171,7 @@
         <v>2050</v>
       </c>
       <c r="F172">
-        <v>0.1668211948277722</v>
+        <v>0.1666540263579375</v>
       </c>
     </row>
     <row r="173">
@@ -5479,7 +5479,7 @@
         <v>2050</v>
       </c>
       <c r="F183">
-        <v>0.08671258408835963</v>
+        <v>0.08662569099295631</v>
       </c>
     </row>
     <row r="184">
@@ -5535,7 +5535,7 @@
         <v>2050</v>
       </c>
       <c r="F185">
-        <v>0.6659696282424172</v>
+        <v>0.6659083560325868</v>
       </c>
     </row>
     <row r="186">
@@ -5815,7 +5815,7 @@
         <v>2050</v>
       </c>
       <c r="F195">
-        <v>0.6804212598293454</v>
+        <v>0.679739422123015</v>
       </c>
     </row>
     <row r="196">
@@ -5843,7 +5843,7 @@
         <v>2050</v>
       </c>
       <c r="F196">
-        <v>0.2462598590314732</v>
+        <v>0.2460130865283839</v>
       </c>
     </row>
     <row r="197">
@@ -6319,7 +6319,7 @@
         <v>2050</v>
       </c>
       <c r="F213">
-        <v>9.910009610098246E-05</v>
+        <v>9.900078970623581E-05</v>
       </c>
     </row>
     <row r="214">
@@ -7495,7 +7495,7 @@
         <v>2050</v>
       </c>
       <c r="F255">
-        <v>1.63515158566621</v>
+        <v>1.633513030152891</v>
       </c>
     </row>
     <row r="256">
@@ -7523,7 +7523,7 @@
         <v>2050</v>
       </c>
       <c r="F256">
-        <v>0.08221901745083056</v>
+        <v>0.08213662727641204</v>
       </c>
     </row>
     <row r="257">
@@ -7663,7 +7663,7 @@
         <v>2050</v>
       </c>
       <c r="F261">
-        <v>0.3220753123281929</v>
+        <v>0.3217525665452662</v>
       </c>
     </row>
     <row r="262">
@@ -7691,7 +7691,7 @@
         <v>2050</v>
       </c>
       <c r="F262">
-        <v>0.004369126531203558</v>
+        <v>0.004364748309374553</v>
       </c>
     </row>
     <row r="263">
@@ -7831,7 +7831,7 @@
         <v>2050</v>
       </c>
       <c r="F267">
-        <v>0.9140001863393612</v>
+        <v>0.9130842834606129</v>
       </c>
     </row>
     <row r="268">
@@ -7859,7 +7859,7 @@
         <v>2050</v>
       </c>
       <c r="F268">
-        <v>0.6513970464703484</v>
+        <v>0.6507442933976606</v>
       </c>
     </row>
     <row r="269">
@@ -8167,7 +8167,7 @@
         <v>2050</v>
       </c>
       <c r="F279">
-        <v>0.7000532429697606</v>
+        <v>0.6993517324119989</v>
       </c>
     </row>
     <row r="280">
@@ -8195,7 +8195,7 @@
         <v>2050</v>
       </c>
       <c r="F280">
-        <v>1.402092423195323</v>
+        <v>1.400687412008379</v>
       </c>
     </row>
     <row r="281">
@@ -8531,7 +8531,7 @@
         <v>2050</v>
       </c>
       <c r="F292">
-        <v>0.0005560706494259071</v>
+        <v>0.000555513421193125</v>
       </c>
     </row>
     <row r="293">
@@ -8839,7 +8839,7 @@
         <v>2050</v>
       </c>
       <c r="F303">
-        <v>0.04955004805049122</v>
+        <v>0.0495003948531179</v>
       </c>
     </row>
     <row r="304">
@@ -8867,7 +8867,7 @@
         <v>2050</v>
       </c>
       <c r="F304">
-        <v>0.001588773284074021</v>
+        <v>0.001587181203408928</v>
       </c>
     </row>
     <row r="305">
@@ -9175,7 +9175,7 @@
         <v>2050</v>
       </c>
       <c r="F315">
-        <v>0.05906365727618554</v>
+        <v>0.05900447066491653</v>
       </c>
     </row>
     <row r="316">
@@ -9203,7 +9203,7 @@
         <v>2050</v>
       </c>
       <c r="F316">
-        <v>0.05560706494259071</v>
+        <v>0.05555134211931249</v>
       </c>
     </row>
     <row r="317">
@@ -9679,7 +9679,7 @@
         <v>2050</v>
       </c>
       <c r="F333">
-        <v>1.8056037509599</v>
+        <v>1.803794388447616</v>
       </c>
     </row>
     <row r="334">
@@ -9707,7 +9707,7 @@
         <v>2050</v>
       </c>
       <c r="F334">
-        <v>0.7626111763555298</v>
+        <v>0.7618469776362856</v>
       </c>
     </row>
     <row r="335">
@@ -9847,7 +9847,7 @@
         <v>2050</v>
       </c>
       <c r="F339">
-        <v>1.040551009060316</v>
+        <v>1.039508291915476</v>
       </c>
     </row>
     <row r="340">
@@ -9875,7 +9875,7 @@
         <v>2050</v>
       </c>
       <c r="F340">
-        <v>0.07943866420370102</v>
+        <v>0.0793590601704464</v>
       </c>
     </row>
     <row r="341">
@@ -10183,7 +10183,7 @@
         <v>2050</v>
       </c>
       <c r="F351">
-        <v>0.01982001922019649</v>
+        <v>0.01980015794124716</v>
       </c>
     </row>
     <row r="352">
@@ -10883,7 +10883,7 @@
         <v>2050</v>
       </c>
       <c r="F376">
-        <v>0.1191579963055516</v>
+        <v>0.1190385902556696</v>
       </c>
     </row>
     <row r="377">

</xml_diff>